<commit_message>
Docs work No 1
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schar\Desktop\FloatingFace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85177120-7821-4ED6-80C2-B70635829C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626D5683-6A20-4E05-92AD-B65476AE929B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{65A387F2-4D39-4CDA-A8A0-A4AD32069BFB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
   <si>
     <t>Id</t>
   </si>
@@ -62,30 +62,18 @@
     <t>https://www.waveshare.com/st3215-servo.htm?sku=22414</t>
   </si>
   <si>
-    <t>21.99$</t>
-  </si>
-  <si>
     <t>https://www.waveshare.com/product/modules/motors-servos/drivers/bus-servo-adapter-a.htm</t>
   </si>
   <si>
-    <t>4.99$</t>
-  </si>
-  <si>
     <t>ST3215 Waveshare</t>
   </si>
   <si>
     <t>Serial Bus Servo Driver Board</t>
   </si>
   <si>
-    <t>1m 2020 Profile</t>
-  </si>
-  <si>
     <t>link</t>
   </si>
   <si>
-    <t>10,52$</t>
-  </si>
-  <si>
     <t>Note</t>
   </si>
   <si>
@@ -95,29 +83,79 @@
     <t>U-Light Sensor</t>
   </si>
   <si>
-    <t>2,76$</t>
-  </si>
-  <si>
-    <t>https://agelektronik.de/allnet-produkte-new/6696-arduino-sensor-lichtschranken-modul-3pol.html</t>
-  </si>
-  <si>
-    <t>https://www.mtsmagnete.de/neodym-quader-magnete/quader-10mm-19mm/neodym-quadermagnet-10x10x5mm-neodym-beschichtung-grade-n45-magnetisiert-durch-5mm/a-2890/?ReferrerID=13&amp;gad_source=1&amp;gad_campaignid=21249616227&amp;gbraid=0AAAAADwDoowZvOoVUnYe6jItQ3B0ME6E9&amp;gclid=CjwKCAjwvqjOBhAGEiwAngeQnbmSshaGV7x5jKac5awHnQgPc2SYVbYD76EYpkBMAvTYsqUXHywgdxoCo48QAvD_BwE</t>
-  </si>
-  <si>
-    <t>Neodym magnets</t>
-  </si>
-  <si>
     <t>TMC2209 Drivers</t>
   </si>
   <si>
     <t>AS5600 Magnetic Encodes</t>
+  </si>
+  <si>
+    <t>900mm 2020 Profile</t>
+  </si>
+  <si>
+    <t>delta_drive v1.1</t>
+  </si>
+  <si>
+    <t>smallest order qty</t>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t>10x10x5 Neodym magnets</t>
+  </si>
+  <si>
+    <t>Cheaper magnets have not the necessary documentation and polarity</t>
+  </si>
+  <si>
+    <t>ESP32-S3-DevKitC-1</t>
+  </si>
+  <si>
+    <t>TCA9548A</t>
+  </si>
+  <si>
+    <t>MPU 5060</t>
+  </si>
+  <si>
+    <t>NEMA17 0.5Nm</t>
+  </si>
+  <si>
+    <t>already got some</t>
+  </si>
+  <si>
+    <t>1kg ABS</t>
+  </si>
+  <si>
+    <t>https://eu.store.bambulab.com/de/products/abs-filament?id=46963746046300</t>
+  </si>
+  <si>
+    <t>EUR/USD exchange:</t>
+  </si>
+  <si>
+    <t>SUM:</t>
+  </si>
+  <si>
+    <t>all EUR entries</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> all USD entries</t>
+  </si>
+  <si>
+    <t>JLCPCB, see picture on github</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="6">
+    <numFmt numFmtId="6" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    <numFmt numFmtId="169" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="171" formatCode="[$$-409]#,##0.00_ ;\-[$$-409]#,##0.00\ "/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,6 +167,27 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF191919"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -151,15 +210,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -493,18 +566,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95230265-E512-4083-959E-E259C2CF6DF4}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.28515625" customWidth="1"/>
     <col min="2" max="2" width="30.5703125" customWidth="1"/>
     <col min="3" max="3" width="22.140625" customWidth="1"/>
     <col min="4" max="4" width="98.28515625" customWidth="1"/>
-    <col min="5" max="5" width="24.140625" customWidth="1"/>
-    <col min="6" max="6" width="44" customWidth="1"/>
+    <col min="5" max="6" width="24.140625" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -521,10 +594,13 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -534,263 +610,318 @@
       <c r="C2">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="7">
+        <v>5.13</v>
+      </c>
+      <c r="F2" s="7">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E3" s="7">
+        <v>2.99</v>
+      </c>
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="7">
+        <v>4.99</v>
+      </c>
+      <c r="F4" s="7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <v>4</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E5" s="7">
+        <v>10.52</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="E6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2">
+        <v>7.16</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C7">
         <v>3</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E7" s="2">
+        <v>2.76</v>
+      </c>
+      <c r="F7" s="2">
+        <v>5.59</v>
+      </c>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8">
         <v>5</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2">
+        <v>7.57</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2">
+        <v>9</v>
+      </c>
+      <c r="F9" s="4">
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="8">
+        <v>7</v>
+      </c>
+      <c r="F10" s="9">
+        <v>3.3</v>
+      </c>
+      <c r="G10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="8">
+        <v>7.77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="8">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="8">
+        <v>1.17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28">
+      <c r="B15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29">
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30">
+      <c r="E15" s="2">
+        <v>25.99</v>
+      </c>
+    </row>
+    <row r="19" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D19" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="2">
+        <f>SUM(E6:E9)+E15</f>
+        <v>52.480000000000004</v>
+      </c>
+      <c r="F19" s="2">
+        <f>F9+F7</f>
+        <v>7.15</v>
+      </c>
+      <c r="G19" s="2">
+        <f>SUM(E19:F19)</f>
+        <v>59.63</v>
+      </c>
+    </row>
+    <row r="20" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="10">
+        <f>SUM(E2:E5)</f>
+        <v>23.630000000000003</v>
+      </c>
+      <c r="F20" s="7">
+        <f>F10+F4+F2</f>
+        <v>9.9500000000000011</v>
+      </c>
+      <c r="G20" s="7">
+        <f>SUM(E20:F20)</f>
+        <v>33.580000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="E22" s="6" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31">
+      <c r="F22">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="4:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="E24" s="11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>37</v>
+    <row r="25" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="E25" s="7">
+        <f>G20+G19*F22</f>
+        <v>102.15450000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="H26" s="5">
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>
@@ -798,8 +929,17 @@
     <hyperlink ref="D5" r:id="rId1" xr:uid="{23658DED-FD76-4C24-A5E2-91FF13C44E8E}"/>
     <hyperlink ref="D7" r:id="rId2" xr:uid="{6BDAC8F8-1877-4CB3-8247-CED8789400D0}"/>
     <hyperlink ref="D8" r:id="rId3" xr:uid="{A90ECC61-BBC8-473F-B0B6-ED98E816B181}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{0162EDAC-20A2-4D97-88C3-932115946167}"/>
+    <hyperlink ref="D9" r:id="rId5" xr:uid="{2B579566-7351-4001-B467-7AE14D1BE309}"/>
+    <hyperlink ref="D2" r:id="rId6" xr:uid="{1F54F4FE-D1A8-43DA-9E75-29C07D09CB93}"/>
+    <hyperlink ref="D3" r:id="rId7" xr:uid="{29FAF547-01C9-4098-BC8F-2AF279ECC382}"/>
+    <hyperlink ref="D4" r:id="rId8" xr:uid="{D5B3F6C8-1BF5-4978-B414-95696F39BE25}"/>
+    <hyperlink ref="D11" r:id="rId9" xr:uid="{27BB0205-0FC8-47FE-95DD-00E7D155E4A2}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{2C741165-C0AF-4DBD-8D7F-4C82C59D6E27}"/>
+    <hyperlink ref="D13" r:id="rId11" xr:uid="{07AC4F73-ED05-45E1-9E5D-CFED507062F3}"/>
+    <hyperlink ref="D15" r:id="rId12" xr:uid="{77FFE69D-C4F4-4CF6-B161-9CAD8E3D9D3F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>